<commit_message>
Variado, PWS log de errores, workflow modificado, docker html
</commit_message>
<xml_diff>
--- a/Documentos/EjemploExcel.xlsx
+++ b/Documentos/EjemploExcel.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30128"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Descargas\Programas\scripts\Powershell\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9F294047-A048-4C65-B8D5-90679DED4259}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DCFF5B7D-4411-41B4-9B06-DE02091EDC27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="84">
   <si>
     <t>NIVEL 1</t>
   </si>
@@ -62,27 +63,195 @@
     <t>G04</t>
   </si>
   <si>
+    <t>01. A</t>
+  </si>
+  <si>
+    <t>01.01. AA</t>
+  </si>
+  <si>
+    <t>01.01.01. AAA</t>
+  </si>
+  <si>
+    <t>RW</t>
+  </si>
+  <si>
+    <t>RO</t>
+  </si>
+  <si>
+    <t>01.01.02. AAB</t>
+  </si>
+  <si>
+    <t>01.01.03. AAC</t>
+  </si>
+  <si>
+    <t>01.02. AB</t>
+  </si>
+  <si>
+    <t>01.02.01. ABA</t>
+  </si>
+  <si>
+    <t>01.02.02. ABB</t>
+  </si>
+  <si>
+    <t>01.02.03. ABC</t>
+  </si>
+  <si>
+    <t>01.02.04. ABD</t>
+  </si>
+  <si>
+    <t>01.02.04.01. ABDA</t>
+  </si>
+  <si>
+    <t>01.02.04.02. ABDB</t>
+  </si>
+  <si>
+    <t>01.02.05. ABE</t>
+  </si>
+  <si>
+    <t>01.02.06. ABF</t>
+  </si>
+  <si>
+    <t>01.03. AC</t>
+  </si>
+  <si>
+    <t>01.03.01. ACA</t>
+  </si>
+  <si>
+    <t>01.03.02. ACB</t>
+  </si>
+  <si>
+    <t>01.03.03. ACC</t>
+  </si>
+  <si>
+    <t>01.03.04. ACD</t>
+  </si>
+  <si>
+    <t>01.04. AD</t>
+  </si>
+  <si>
+    <t>01.04.01. ADA</t>
+  </si>
+  <si>
+    <t>01.04.02. ADB</t>
+  </si>
+  <si>
+    <t>01.05. AE</t>
+  </si>
+  <si>
+    <t>01.06. AF</t>
+  </si>
+  <si>
+    <t>02. B</t>
+  </si>
+  <si>
+    <t>02.01. BA</t>
+  </si>
+  <si>
+    <t>02.02. BB</t>
+  </si>
+  <si>
+    <t>02.03. BC</t>
+  </si>
+  <si>
+    <t>02.03.01. BCA</t>
+  </si>
+  <si>
+    <t>02.03.02. BCB</t>
+  </si>
+  <si>
+    <t>02.03.03. BCC</t>
+  </si>
+  <si>
+    <t>02.03.04. BCD</t>
+  </si>
+  <si>
+    <t>02.04. BD</t>
+  </si>
+  <si>
+    <t>02.04.01. BDA</t>
+  </si>
+  <si>
+    <t>02.04.02. BDB</t>
+  </si>
+  <si>
+    <t>BDBA</t>
+  </si>
+  <si>
+    <t>BDBB</t>
+  </si>
+  <si>
+    <t>BDBC</t>
+  </si>
+  <si>
+    <t>02.05. BE</t>
+  </si>
+  <si>
+    <t>02.05.01. BEA</t>
+  </si>
+  <si>
+    <t>02.05.02. BEB</t>
+  </si>
+  <si>
+    <t>02.05.03. BEC</t>
+  </si>
+  <si>
+    <t>02.05.04. BED</t>
+  </si>
+  <si>
+    <t>02.05.05. BEE</t>
+  </si>
+  <si>
+    <t>02.06. BF</t>
+  </si>
+  <si>
+    <t>02.06.01. BFA</t>
+  </si>
+  <si>
+    <t>02.06.02. BFB</t>
+  </si>
+  <si>
+    <t>02.07. BG</t>
+  </si>
+  <si>
+    <t>02.08. BH</t>
+  </si>
+  <si>
+    <t>02.09. BI</t>
+  </si>
+  <si>
+    <t>02.10. BJ</t>
+  </si>
+  <si>
+    <t>02.11. BK</t>
+  </si>
+  <si>
+    <t>03. C</t>
+  </si>
+  <si>
+    <t>03.01. CA</t>
+  </si>
+  <si>
+    <t>03.02. CB</t>
+  </si>
+  <si>
+    <t>03.03. CC</t>
+  </si>
+  <si>
+    <t>03.03.01. CCA</t>
+  </si>
+  <si>
+    <t>03.03.02. CCB</t>
+  </si>
+  <si>
+    <t>03.04. CD</t>
+  </si>
+  <si>
+    <t>NIVEL 5</t>
+  </si>
+  <si>
     <t>01 A</t>
   </si>
   <si>
-    <t>01.01 AA</t>
-  </si>
-  <si>
-    <t>01.01.01 AAA</t>
-  </si>
-  <si>
-    <t>RW</t>
-  </si>
-  <si>
-    <t>RO</t>
-  </si>
-  <si>
-    <t>01.01.02 AAB</t>
-  </si>
-  <si>
-    <t>01.01.03 AAC</t>
-  </si>
-  <si>
     <t>01.02 AB</t>
   </si>
   <si>
@@ -116,133 +285,10 @@
     <t>01.03.01 ACA</t>
   </si>
   <si>
-    <t>01.03.02 ACB</t>
-  </si>
-  <si>
-    <t>01.03.03 ACC</t>
-  </si>
-  <si>
-    <t>01.03.04 ACD</t>
-  </si>
-  <si>
-    <t>01.04 AD</t>
-  </si>
-  <si>
-    <t>01.04.01 ADA</t>
-  </si>
-  <si>
-    <t>01.04.02 ADB</t>
-  </si>
-  <si>
-    <t>01.05 AE</t>
-  </si>
-  <si>
-    <t>01.06 AF</t>
-  </si>
-  <si>
-    <t>02 B</t>
-  </si>
-  <si>
-    <t>02.01 BA</t>
-  </si>
-  <si>
-    <t>02.02 BB</t>
-  </si>
-  <si>
-    <t>02.03 BC</t>
-  </si>
-  <si>
-    <t>02.03.01 BCA</t>
-  </si>
-  <si>
-    <t>02.03.02 BCB</t>
-  </si>
-  <si>
-    <t>02.03.03 BCC</t>
-  </si>
-  <si>
-    <t>02.03.04 BCD</t>
-  </si>
-  <si>
-    <t>02.04 BD</t>
-  </si>
-  <si>
-    <t>02.04.01 BDA</t>
-  </si>
-  <si>
-    <t>02.04.02 BDB</t>
-  </si>
-  <si>
-    <t>BDBA</t>
-  </si>
-  <si>
-    <t>BDBB</t>
-  </si>
-  <si>
-    <t>BDBC</t>
-  </si>
-  <si>
-    <t>02.05 BE</t>
-  </si>
-  <si>
-    <t>02.05.01 BEA</t>
-  </si>
-  <si>
-    <t>02.05.02 BEB</t>
-  </si>
-  <si>
-    <t>02.05.03 BEC</t>
-  </si>
-  <si>
-    <t>02.05.04: BED</t>
-  </si>
-  <si>
-    <t>02.05.05: BEE</t>
-  </si>
-  <si>
-    <t>02.06. BF</t>
-  </si>
-  <si>
-    <t>02.06.01: BFA</t>
-  </si>
-  <si>
-    <t>02.06.01: BFB</t>
-  </si>
-  <si>
-    <t>02.07: BG</t>
-  </si>
-  <si>
-    <t>02.08. BH</t>
-  </si>
-  <si>
-    <t>02.09 BI</t>
-  </si>
-  <si>
-    <t>02.10 BJ</t>
-  </si>
-  <si>
-    <t>02.11 BK</t>
-  </si>
-  <si>
-    <t>03 C</t>
-  </si>
-  <si>
-    <t>03.01 CA</t>
-  </si>
-  <si>
-    <t>03.02 CB</t>
-  </si>
-  <si>
-    <t>03.03 CC</t>
-  </si>
-  <si>
-    <t>03.03.01 CCA</t>
-  </si>
-  <si>
-    <t>03.03.02 CCB</t>
-  </si>
-  <si>
-    <t>03.04 CD</t>
+    <t>01.03.01.01 ACAA</t>
+  </si>
+  <si>
+    <t>01.03.01.01.01 ACAAA</t>
   </si>
 </sst>
 </file>
@@ -451,13 +497,13 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -823,28 +869,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="E1" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="17" t="s">
+      <c r="F1" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="17" t="s">
+      <c r="G1" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="17" t="s">
+      <c r="H1" s="15" t="s">
         <v>7</v>
       </c>
     </row>
@@ -855,60 +901,60 @@
       <c r="B2" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="15"/>
-      <c r="E2" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="G2" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="H2" s="16" t="s">
+      <c r="D2" s="16"/>
+      <c r="E2" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" s="17" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="23"/>
       <c r="B3" s="18"/>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="15"/>
-      <c r="E3" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="H3" s="16" t="s">
+      <c r="D3" s="16"/>
+      <c r="E3" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="H3" s="17" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="23"/>
       <c r="B4" s="18"/>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="15"/>
-      <c r="E4" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="H4" s="16" t="s">
+      <c r="D4" s="16"/>
+      <c r="E4" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="H4" s="17" t="s">
         <v>12</v>
       </c>
     </row>
@@ -917,52 +963,52 @@
       <c r="B5" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="15"/>
-      <c r="E5" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G5" s="16"/>
-      <c r="H5" s="16"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" s="17"/>
+      <c r="H5" s="17"/>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="23"/>
       <c r="B6" s="18"/>
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="15"/>
-      <c r="E6" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G6" s="16"/>
-      <c r="H6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" s="17"/>
+      <c r="H6" s="17"/>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="23"/>
       <c r="B7" s="18"/>
-      <c r="C7" s="15" t="s">
+      <c r="C7" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="15"/>
-      <c r="E7" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="G7" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="H7" s="16" t="s">
+      <c r="D7" s="16"/>
+      <c r="E7" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="H7" s="17" t="s">
         <v>12</v>
       </c>
     </row>
@@ -972,19 +1018,19 @@
       <c r="C8" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="15" t="s">
+      <c r="D8" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="E8" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G8" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="H8" s="16" t="s">
+      <c r="E8" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="H8" s="17" t="s">
         <v>11</v>
       </c>
     </row>
@@ -992,59 +1038,59 @@
       <c r="A9" s="23"/>
       <c r="B9" s="18"/>
       <c r="C9" s="18"/>
-      <c r="D9" s="15" t="s">
+      <c r="D9" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="E9" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F9" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G9" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="H9" s="16" t="s">
+      <c r="E9" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G9" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="H9" s="17" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" s="23"/>
       <c r="B10" s="18"/>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="D10" s="15"/>
-      <c r="E10" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F10" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G10" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="H10" s="16" t="s">
+      <c r="D10" s="16"/>
+      <c r="E10" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="H10" s="17" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="23"/>
       <c r="B11" s="18"/>
-      <c r="C11" s="15" t="s">
+      <c r="C11" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="15"/>
-      <c r="E11" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F11" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="G11" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="H11" s="16" t="s">
+      <c r="D11" s="16"/>
+      <c r="E11" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F11" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="H11" s="17" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1053,138 +1099,138 @@
       <c r="B12" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="C12" s="15" t="s">
+      <c r="C12" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="15"/>
-      <c r="E12" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F12" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="G12" s="16"/>
-      <c r="H12" s="16"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F12" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="G12" s="17"/>
+      <c r="H12" s="17"/>
     </row>
     <row r="13" spans="1:8">
       <c r="A13" s="23"/>
       <c r="B13" s="18"/>
-      <c r="C13" s="15" t="s">
+      <c r="C13" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="D13" s="15"/>
-      <c r="E13" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F13" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="G13" s="16"/>
-      <c r="H13" s="16"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F13" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="G13" s="17"/>
+      <c r="H13" s="17"/>
     </row>
     <row r="14" spans="1:8">
       <c r="A14" s="23"/>
       <c r="B14" s="18"/>
-      <c r="C14" s="15" t="s">
+      <c r="C14" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="D14" s="15"/>
-      <c r="E14" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F14" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G14" s="16"/>
-      <c r="H14" s="16"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F14" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G14" s="17"/>
+      <c r="H14" s="17"/>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="23"/>
       <c r="B15" s="18"/>
-      <c r="C15" s="15" t="s">
+      <c r="C15" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="D15" s="15"/>
-      <c r="E15" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F15" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G15" s="16"/>
-      <c r="H15" s="16"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F15" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G15" s="17"/>
+      <c r="H15" s="17"/>
     </row>
     <row r="16" spans="1:8">
       <c r="A16" s="23"/>
       <c r="B16" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="C16" s="15" t="s">
+      <c r="C16" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="D16" s="15"/>
-      <c r="E16" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F16" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G16" s="16"/>
-      <c r="H16" s="16"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F16" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G16" s="17"/>
+      <c r="H16" s="17"/>
     </row>
     <row r="17" spans="1:8">
       <c r="A17" s="23"/>
       <c r="B17" s="18"/>
-      <c r="C17" s="15" t="s">
+      <c r="C17" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="D17" s="15"/>
-      <c r="E17" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F17" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G17" s="16"/>
-      <c r="H17" s="16"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F17" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G17" s="17"/>
+      <c r="H17" s="17"/>
     </row>
     <row r="18" spans="1:8">
       <c r="A18" s="23"/>
-      <c r="B18" s="15" t="s">
+      <c r="B18" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="C18" s="15"/>
-      <c r="D18" s="15"/>
-      <c r="E18" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F18" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="G18" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="H18" s="16" t="s">
+      <c r="C18" s="16"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F18" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="G18" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="H18" s="17" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="19" spans="1:8">
       <c r="A19" s="23"/>
-      <c r="B19" s="15" t="s">
+      <c r="B19" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="C19" s="15"/>
-      <c r="D19" s="15"/>
-      <c r="E19" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F19" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="G19" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="H19" s="16" t="s">
+      <c r="C19" s="16"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F19" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="G19" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="H19" s="17" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1192,41 +1238,41 @@
       <c r="A20" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="B20" s="15" t="s">
+      <c r="B20" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="C20" s="15"/>
-      <c r="D20" s="15"/>
-      <c r="E20" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F20" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G20" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="H20" s="16" t="s">
+      <c r="C20" s="16"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F20" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G20" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="H20" s="17" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="21" spans="1:8">
       <c r="A21" s="20"/>
-      <c r="B21" s="15" t="s">
+      <c r="B21" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="C21" s="15"/>
-      <c r="D21" s="15"/>
-      <c r="E21" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F21" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G21" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="H21" s="16" t="s">
+      <c r="C21" s="16"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F21" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G21" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="H21" s="17" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1235,76 +1281,76 @@
       <c r="B22" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="C22" s="15" t="s">
+      <c r="C22" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="D22" s="15"/>
-      <c r="E22" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F22" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G22" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="H22" s="16"/>
+      <c r="D22" s="16"/>
+      <c r="E22" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F22" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G22" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="H22" s="17"/>
     </row>
     <row r="23" spans="1:8">
       <c r="A23" s="20"/>
       <c r="B23" s="18"/>
-      <c r="C23" s="15" t="s">
+      <c r="C23" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="D23" s="15"/>
-      <c r="E23" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F23" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G23" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="H23" s="16"/>
+      <c r="D23" s="16"/>
+      <c r="E23" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F23" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G23" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="H23" s="17"/>
     </row>
     <row r="24" spans="1:8">
       <c r="A24" s="20"/>
       <c r="B24" s="18"/>
-      <c r="C24" s="15" t="s">
+      <c r="C24" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="D24" s="15"/>
-      <c r="E24" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F24" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G24" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="H24" s="16" t="s">
+      <c r="D24" s="16"/>
+      <c r="E24" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F24" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G24" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="H24" s="17" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="25" spans="1:8">
       <c r="A25" s="20"/>
       <c r="B25" s="18"/>
-      <c r="C25" s="15" t="s">
+      <c r="C25" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="D25" s="15"/>
-      <c r="E25" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F25" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G25" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="H25" s="16" t="s">
+      <c r="D25" s="16"/>
+      <c r="E25" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F25" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G25" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="H25" s="17" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1313,18 +1359,18 @@
       <c r="B26" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="C26" s="15" t="s">
+      <c r="C26" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="D26" s="15"/>
-      <c r="E26" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F26" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G26" s="16"/>
-      <c r="H26" s="16"/>
+      <c r="D26" s="16"/>
+      <c r="E26" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F26" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G26" s="17"/>
+      <c r="H26" s="17"/>
     </row>
     <row r="27" spans="1:8">
       <c r="A27" s="20"/>
@@ -1332,253 +1378,253 @@
       <c r="C27" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="D27" s="15" t="s">
+      <c r="D27" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="E27" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F27" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G27" s="16"/>
-      <c r="H27" s="16"/>
+      <c r="E27" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F27" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G27" s="17"/>
+      <c r="H27" s="17"/>
     </row>
     <row r="28" spans="1:8">
       <c r="A28" s="20"/>
       <c r="B28" s="18"/>
       <c r="C28" s="18"/>
-      <c r="D28" s="15" t="s">
+      <c r="D28" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="E28" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F28" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G28" s="16"/>
-      <c r="H28" s="16"/>
+      <c r="E28" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F28" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G28" s="17"/>
+      <c r="H28" s="17"/>
     </row>
     <row r="29" spans="1:8">
       <c r="A29" s="20"/>
       <c r="B29" s="18"/>
       <c r="C29" s="18"/>
-      <c r="D29" s="15" t="s">
+      <c r="D29" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="E29" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F29" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G29" s="16"/>
-      <c r="H29" s="16"/>
+      <c r="E29" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F29" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G29" s="17"/>
+      <c r="H29" s="17"/>
     </row>
     <row r="30" spans="1:8">
       <c r="A30" s="20"/>
       <c r="B30" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="C30" s="15" t="s">
+      <c r="C30" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="D30" s="15"/>
-      <c r="E30" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F30" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G30" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="H30" s="16"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F30" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G30" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="H30" s="17"/>
     </row>
     <row r="31" spans="1:8">
       <c r="A31" s="20"/>
       <c r="B31" s="18"/>
-      <c r="C31" s="15" t="s">
+      <c r="C31" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="D31" s="15"/>
-      <c r="E31" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F31" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G31" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="H31" s="16"/>
+      <c r="D31" s="16"/>
+      <c r="E31" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F31" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G31" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="H31" s="17"/>
     </row>
     <row r="32" spans="1:8">
       <c r="A32" s="20"/>
       <c r="B32" s="18"/>
-      <c r="C32" s="15" t="s">
+      <c r="C32" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="D32" s="15"/>
-      <c r="E32" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F32" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G32" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="H32" s="16"/>
+      <c r="D32" s="16"/>
+      <c r="E32" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F32" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G32" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="H32" s="17"/>
     </row>
     <row r="33" spans="1:8">
       <c r="A33" s="20"/>
       <c r="B33" s="18"/>
-      <c r="C33" s="15" t="s">
+      <c r="C33" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="D33" s="15"/>
-      <c r="E33" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F33" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G33" s="16"/>
-      <c r="H33" s="16"/>
+      <c r="D33" s="16"/>
+      <c r="E33" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F33" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G33" s="17"/>
+      <c r="H33" s="17"/>
     </row>
     <row r="34" spans="1:8">
       <c r="A34" s="20"/>
       <c r="B34" s="18"/>
-      <c r="C34" s="15" t="s">
+      <c r="C34" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="D34" s="15"/>
-      <c r="E34" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F34" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G34" s="16"/>
-      <c r="H34" s="16"/>
+      <c r="D34" s="16"/>
+      <c r="E34" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F34" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G34" s="17"/>
+      <c r="H34" s="17"/>
     </row>
     <row r="35" spans="1:8">
       <c r="A35" s="20"/>
       <c r="B35" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="C35" s="15" t="s">
+      <c r="C35" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="D35" s="15"/>
-      <c r="E35" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F35" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G35" s="16"/>
-      <c r="H35" s="16"/>
+      <c r="D35" s="16"/>
+      <c r="E35" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F35" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G35" s="17"/>
+      <c r="H35" s="17"/>
     </row>
     <row r="36" spans="1:8">
       <c r="A36" s="20"/>
       <c r="B36" s="18"/>
-      <c r="C36" s="15" t="s">
+      <c r="C36" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="D36" s="15"/>
-      <c r="E36" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F36" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G36" s="16"/>
-      <c r="H36" s="16"/>
+      <c r="D36" s="16"/>
+      <c r="E36" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F36" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G36" s="17"/>
+      <c r="H36" s="17"/>
     </row>
     <row r="37" spans="1:8">
       <c r="A37" s="20"/>
-      <c r="B37" s="15" t="s">
+      <c r="B37" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="C37" s="15"/>
-      <c r="D37" s="15"/>
-      <c r="E37" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F37" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G37" s="16"/>
-      <c r="H37" s="16"/>
+      <c r="C37" s="16"/>
+      <c r="D37" s="16"/>
+      <c r="E37" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F37" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G37" s="17"/>
+      <c r="H37" s="17"/>
     </row>
     <row r="38" spans="1:8">
       <c r="A38" s="20"/>
-      <c r="B38" s="15" t="s">
+      <c r="B38" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="C38" s="15"/>
-      <c r="D38" s="15"/>
-      <c r="E38" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F38" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G38" s="16"/>
-      <c r="H38" s="16"/>
+      <c r="C38" s="16"/>
+      <c r="D38" s="16"/>
+      <c r="E38" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F38" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G38" s="17"/>
+      <c r="H38" s="17"/>
     </row>
     <row r="39" spans="1:8">
       <c r="A39" s="20"/>
-      <c r="B39" s="15" t="s">
+      <c r="B39" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="C39" s="15"/>
-      <c r="D39" s="15"/>
-      <c r="E39" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F39" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G39" s="16"/>
-      <c r="H39" s="16"/>
+      <c r="C39" s="16"/>
+      <c r="D39" s="16"/>
+      <c r="E39" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F39" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G39" s="17"/>
+      <c r="H39" s="17"/>
     </row>
     <row r="40" spans="1:8">
       <c r="A40" s="20"/>
-      <c r="B40" s="15" t="s">
+      <c r="B40" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="C40" s="15"/>
-      <c r="D40" s="15"/>
-      <c r="E40" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F40" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G40" s="16"/>
-      <c r="H40" s="16"/>
+      <c r="C40" s="16"/>
+      <c r="D40" s="16"/>
+      <c r="E40" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F40" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G40" s="17"/>
+      <c r="H40" s="17"/>
     </row>
     <row r="41" spans="1:8">
       <c r="A41" s="21"/>
-      <c r="B41" s="15" t="s">
+      <c r="B41" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="C41" s="15"/>
-      <c r="D41" s="15"/>
-      <c r="E41" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F41" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G41" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="H41" s="16" t="s">
+      <c r="C41" s="16"/>
+      <c r="D41" s="16"/>
+      <c r="E41" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F41" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G41" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="H41" s="17" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1586,41 +1632,41 @@
       <c r="A42" s="22" t="s">
         <v>62</v>
       </c>
-      <c r="B42" s="15" t="s">
+      <c r="B42" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="C42" s="15"/>
-      <c r="D42" s="15"/>
-      <c r="E42" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F42" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G42" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="H42" s="16" t="s">
+      <c r="C42" s="16"/>
+      <c r="D42" s="16"/>
+      <c r="E42" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F42" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G42" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="H42" s="17" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="43" spans="1:8">
       <c r="A43" s="22"/>
-      <c r="B43" s="15" t="s">
+      <c r="B43" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="C43" s="15"/>
-      <c r="D43" s="15"/>
-      <c r="E43" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F43" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G43" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="H43" s="16" t="s">
+      <c r="C43" s="16"/>
+      <c r="D43" s="16"/>
+      <c r="E43" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F43" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G43" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="H43" s="17" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1629,58 +1675,58 @@
       <c r="B44" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="C44" s="15" t="s">
+      <c r="C44" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="D44" s="15"/>
-      <c r="E44" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F44" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G44" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="H44" s="16" t="s">
+      <c r="D44" s="16"/>
+      <c r="E44" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F44" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G44" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="H44" s="17" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="45" spans="1:8">
       <c r="A45" s="22"/>
       <c r="B45" s="18"/>
-      <c r="C45" s="15" t="s">
+      <c r="C45" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="D45" s="15"/>
-      <c r="E45" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F45" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G45" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="H45" s="16" t="s">
+      <c r="D45" s="16"/>
+      <c r="E45" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F45" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G45" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="H45" s="17" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="46" spans="1:8">
       <c r="A46" s="22"/>
-      <c r="B46" s="15" t="s">
+      <c r="B46" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="C46" s="15"/>
-      <c r="D46" s="15"/>
-      <c r="E46" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F46" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G46" s="16"/>
-      <c r="H46" s="16"/>
+      <c r="C46" s="16"/>
+      <c r="D46" s="16"/>
+      <c r="E46" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F46" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G46" s="17"/>
+      <c r="H46" s="17"/>
     </row>
     <row r="47" spans="1:8">
       <c r="A47" s="13"/>
@@ -2473,4 +2519,341 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF0C8392-49B2-4846-9E1D-727C1E85A943}">
+  <dimension ref="A1:I19"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="14.85546875" customWidth="1"/>
+    <col min="2" max="2" width="16.28515625" customWidth="1"/>
+    <col min="3" max="3" width="16.7109375" customWidth="1"/>
+    <col min="4" max="5" width="21" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="11.5703125" customWidth="1"/>
+    <col min="8" max="8" width="11.42578125" customWidth="1"/>
+    <col min="9" max="9" width="11" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="F1" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="15" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" s="23" t="s">
+        <v>70</v>
+      </c>
+      <c r="B2" s="18"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" s="23"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="17"/>
+      <c r="G3" s="17"/>
+      <c r="H3" s="17"/>
+      <c r="I3" s="17"/>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" s="23"/>
+      <c r="B4" s="18"/>
+      <c r="C4" s="16"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="17"/>
+      <c r="G4" s="17"/>
+      <c r="H4" s="17"/>
+      <c r="I4" s="17"/>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" s="23"/>
+      <c r="B5" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="D5" s="16"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="H5" s="17"/>
+      <c r="I5" s="17"/>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" s="23"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="16" t="s">
+        <v>73</v>
+      </c>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="H6" s="17"/>
+      <c r="I6" s="17"/>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" s="23"/>
+      <c r="B7" s="18"/>
+      <c r="C7" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="H7" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="I7" s="17" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" s="23"/>
+      <c r="B8" s="18"/>
+      <c r="C8" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="D8" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="E8" s="16"/>
+      <c r="F8" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="H8" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="I8" s="17" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" s="23"/>
+      <c r="B9" s="18"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="E9" s="16"/>
+      <c r="F9" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="G9" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="H9" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="I9" s="17" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" s="23"/>
+      <c r="B10" s="18"/>
+      <c r="C10" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="G10" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="H10" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="I10" s="17" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" s="23"/>
+      <c r="B11" s="18"/>
+      <c r="C11" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="H11" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="I11" s="17" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" s="23"/>
+      <c r="B12" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="C12" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="D12" s="16" t="s">
+        <v>82</v>
+      </c>
+      <c r="E12" s="16" t="s">
+        <v>83</v>
+      </c>
+      <c r="F12" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="G12" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="H12" s="17"/>
+      <c r="I12" s="17" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" s="23"/>
+      <c r="B13" s="18"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="17"/>
+      <c r="H13" s="17"/>
+      <c r="I13" s="17"/>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" s="23"/>
+      <c r="B14" s="18"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="17"/>
+      <c r="H14" s="17"/>
+      <c r="I14" s="17"/>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15" s="23"/>
+      <c r="B15" s="18"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="17"/>
+      <c r="H15" s="17"/>
+      <c r="I15" s="17"/>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16" s="23"/>
+      <c r="B16" s="18"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="17"/>
+      <c r="G16" s="17"/>
+      <c r="H16" s="17"/>
+      <c r="I16" s="17"/>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" s="23"/>
+      <c r="B17" s="18"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="17"/>
+      <c r="I17" s="17"/>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" s="23"/>
+      <c r="B18" s="16"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="17"/>
+      <c r="I18" s="17"/>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19" s="23"/>
+      <c r="B19" s="16"/>
+      <c r="C19" s="16"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="16"/>
+      <c r="F19" s="17"/>
+      <c r="G19" s="17"/>
+      <c r="H19" s="17"/>
+      <c r="I19" s="17"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A2:A19"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="B5:B11"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="B12:B15"/>
+    <mergeCell ref="B16:B17"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>